<commit_message>
chore(sync): đồng bộ tài liệu Luận văn, Meeting 4-5, GitHub Pages và phân hệ tái lập PIGuard ACL 2025
</commit_message>
<xml_diff>
--- a/Final-Report/reports/PI_GUARD_PROCESS_REPORT.xlsx
+++ b/Final-Report/reports/PI_GUARD_PROCESS_REPORT.xlsx
@@ -854,7 +854,7 @@
         <is>
           <t>Hoàn thiện Report No.4:
 - Đo lường chỉ số F1, FPR trên CPU.
-- Kiểm toán kết quả nén ONNX INT8.
+- Đánh giá Adversarial Robustness &amp; tối ưu ngưỡng.
 - Nộp Report No.4 cho GVHD.</t>
         </is>
       </c>
@@ -1022,7 +1022,7 @@
         <is>
           <t>Chuẩn bị Hội Đồng 1:
 - Đóng gói tài liệu trích xuất đặc trưng.
-- Kiểm thử chéo mô hình Baseline vs ONNX.
+- Kiểm thử chéo Baseline vs Transformer.
 - Tham gia tổng duyệt demo.</t>
         </is>
       </c>
@@ -1074,7 +1074,7 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Lượng hóa động ONNX INT8 Runtime để tối ưu độ trễ P95 &lt; 30ms trên CPU.</t>
+          <t>Tối ưu hóa pipeline suy luận Transformer và đánh giá độ bền đối kháng Adversarial Robustness.</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -1156,24 +1156,24 @@
       </c>
       <c r="P8" s="6" t="inlineStr">
         <is>
-          <t>Lượng hóa ONNX INT8:
-- Xuất mô hình sang ONNX Runtime.
-- Áp dụng dynamic INT8 quantization.
-- Đạt độ trễ P95 &lt; 30ms trên CPU. Nộp R4.</t>
+          <t>Tối ưu hóa suy luận &amp; Độ bền:
+- Tối ưu hóa suy luận Transformer trên CPU.
+- Đánh giá độ bền đối kháng (Leetspeak, Base64).
+- Đạt độ trễ thấp trên CPU. Nộp R4.</t>
         </is>
       </c>
       <c r="Q8" s="6" t="inlineStr">
         <is>
-          <t>Tích hợp Engine ONNX:
-- Viết wrapper suy luận ONNX cho API.
-- Tối ưu hóa đa luồng CPU (OMP_NUM_THREADS).
+          <t>Tích hợp Transformer Engine:
+- Viết wrapper suy luận DeBERTa-v3 cho API.
+- Tối ưu hóa pipeline batching &amp; đa luồng CPU.
 - Đo đạc thông lượng xử lý RPS.</t>
         </is>
       </c>
       <c r="R8" s="6" t="inlineStr">
         <is>
           <t>Chuẩn bị Hội Đồng 1:
-- Kiểm thử hiệu năng ONNX trên máy trạm.
+- Kiểm thử hiệu năng Transformer trên CPU.
 - Chuẩn bị slide thực nghiệm Chapter 4.
 - Tổng duyệt phần trình bày AI Model.</t>
         </is>
@@ -1181,8 +1181,8 @@
       <c r="S8" s="6" t="inlineStr">
         <is>
           <t>BÁO CÁO HỘI ĐỒNG 1 (MIDTERM):
-- Trình diễn trực tiếp mô hình ONNX INT8.
-- Chứng minh độ trễ P95 &lt; 30ms trên CPU.
+- Trình diễn trực tiếp mô hình DeBERTa-v3 Guardrail.
+- Chứng minh độ trễ thấp và FPR &lt; 1.5%.
 - Bảo vệ thành công Prototype.</t>
         </is>
       </c>
@@ -1197,7 +1197,7 @@
       <c r="U8" s="6" t="inlineStr">
         <is>
           <t>BÁO CÁO HỘI ĐỒNG FINAL (TỐT NGHIỆP):
-- Trình bày kiến trúc DeBERTa &amp; ONNX INT8.
+- Trình bày kiến trúc Two-Tier Guardrail (TF-IDF + DeBERTa-v3).
 - Trả lời chất vấn chuyên sâu về AI Security.
 - Hoàn thành xuất sắc đồ án.</t>
         </is>
@@ -1308,9 +1308,9 @@
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>Tích hợp ONNX Engine:
-- Kết nối mô hình ONNX INT8 vào API.
-- Thêm tính năng toggle chuyển đổi mô hình.
+          <t>Tích hợp Guardrail Engine:
+- Kết nối mô hình phân loại vào FastAPI.
+- Thêm tính năng toggle chuyển đổi mô hình (TF-IDF / DeBERTa).
 - Tối ưu hóa xử lý lỗi HTTP 400/500.</t>
         </is>
       </c>
@@ -2154,7 +2154,7 @@
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>Fine-tuning DeBERTa-v3, Lượng hóa ONNX INT8, Đánh giá Adversarial &amp; Nộp Report No.4</t>
+          <t>Fine-tuning DeBERTa-v3, Đánh giá Adversarial Robustness &amp; Nộp Report No.4</t>
         </is>
       </c>
       <c r="D24" s="13" t="inlineStr">
@@ -2169,7 +2169,7 @@
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
-          <t>Report No.4 &amp; models/onnx/</t>
+          <t>Report No.4 &amp; models/</t>
         </is>
       </c>
       <c r="G24" s="9" t="inlineStr">

</xml_diff>

<commit_message>
feat(meeting-5-6): cap nhat ket qua Meeting 5, tai lieu chuyen de, bo model thuc nghiem va tai nguyen Meeting 6
</commit_message>
<xml_diff>
--- a/Final-Report/reports/PI_GUARD_PROCESS_REPORT.xlsx
+++ b/Final-Report/reports/PI_GUARD_PROCESS_REPORT.xlsx
@@ -112,7 +112,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -134,11 +134,102 @@
         <color rgb="00B0C4DE"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0C4DE"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0C4DE"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B0C4DE"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0C4DE"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B0C4DE"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00B0C4DE"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0C4DE"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0C4DE"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0C4DE"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0C4DE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0C4DE"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0C4DE"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0C4DE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0C4DE"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D3D3D3"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D3D3D3"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -181,6 +272,12 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -610,32 +707,32 @@
           <t>Phân công nhiệm vụ cốt lõi</t>
         </is>
       </c>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
+      <c r="D4" s="15" t="n"/>
+      <c r="E4" s="15" t="n"/>
+      <c r="F4" s="16" t="n"/>
       <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Tiến độ thực hiện hàng tuần (Tuần 1: 07/09/2026 – Tuần 15: 20/12/2026)</t>
         </is>
       </c>
-      <c r="H4" s="4" t="n"/>
-      <c r="I4" s="4" t="n"/>
-      <c r="J4" s="4" t="n"/>
-      <c r="K4" s="4" t="n"/>
-      <c r="L4" s="4" t="n"/>
-      <c r="M4" s="4" t="n"/>
-      <c r="N4" s="4" t="n"/>
-      <c r="O4" s="4" t="n"/>
-      <c r="P4" s="4" t="n"/>
-      <c r="Q4" s="4" t="n"/>
-      <c r="R4" s="4" t="n"/>
-      <c r="S4" s="4" t="n"/>
-      <c r="T4" s="4" t="n"/>
-      <c r="U4" s="4" t="n"/>
+      <c r="H4" s="15" t="n"/>
+      <c r="I4" s="15" t="n"/>
+      <c r="J4" s="15" t="n"/>
+      <c r="K4" s="15" t="n"/>
+      <c r="L4" s="15" t="n"/>
+      <c r="M4" s="15" t="n"/>
+      <c r="N4" s="15" t="n"/>
+      <c r="O4" s="15" t="n"/>
+      <c r="P4" s="15" t="n"/>
+      <c r="Q4" s="15" t="n"/>
+      <c r="R4" s="15" t="n"/>
+      <c r="S4" s="15" t="n"/>
+      <c r="T4" s="15" t="n"/>
+      <c r="U4" s="16" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="5" t="n"/>
-      <c r="B5" s="5" t="n"/>
+      <c r="A5" s="17" t="n"/>
+      <c r="B5" s="17" t="n"/>
       <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Nhiệm vụ 1</t>
@@ -788,10 +885,10 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Bối cảnh &amp; Phân loại:
-- Soạn thảo Chapter 1 (Introduction).
-- Phân loại Threat Taxonomy (OWASP).
-- Lỗ hổng Von Neumann NLP.</t>
+          <t>Thực hiện Task 3 (Replication Lab):
+- Tải và chạy thực nghiệm 5 mô hình y văn public nguyên bản trong truongnv: PIGuard DeBERTa-v3, Ayub MiniLM, Meta Prompt-Guard, Jain Perplexity, InstructDetector.
+- Đo đạc trên 5 benchmark mở (NotInject, WildGuard, BIPIA).
+- Đối soát số liệu đo đạc khớp bài báo ACL 2025.</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -940,10 +1037,10 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>Threat Model &amp; Attack Surface:
-- Xây dựng sơ đồ NIST AI 100-2e2025.
-- Khóa chặt Attack Surface /v1/chat.
-- Thiết kế kiến trúc bảo vệ 3 lớp.</t>
+          <t>Nghiên cứu Task 1 &amp; 2 (Keys &amp; Attack Vectors):
+- Phân biệt 2 key đồ án: Prompt Injection vs. Jailbreak.
+- Phân tích cách thức hoạt động &amp; bề mặt tấn công 2 kênh: Direct Chat vs. Indirect File/RAG.
+- Khung 5 trục NIST AI 100-2e2025, luồng thực thi và blast radius.</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr">
@@ -1092,10 +1189,10 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>Khảo sát Y văn Guardrail:
-- Đối sánh các trường phái Guardrail.
-- Khảo sát các dòng Target LLMs.
-- Soạn thảo luận giải chọn mô hình.</t>
+          <t>Tìm hiểu cơ chế loại bỏ Encoding:
+- Khảo sát các kỹ thuật mã hóa né tránh: Base64, Hexadecimal, Leetspeak, Rot13, ciphers.
+- Tìm hiểu cơ chế bóc tách chuỗi và chuẩn hóa (Tier-0 Scrubber).
+- Đánh giá ảnh hưởng của encoding làm mù tokenizer mô hình.</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -1244,10 +1341,12 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>Research Questions &amp; Gaps:
-- Soạn thảo 3 Câu hỏi IEEE (RQ1-RQ3).
-- Xác định 3 Gaps &amp; 4 Đóng góp mới.
-- Định vị ranh giới In-scope/Out-of-scope.</t>
+          <t>Nghiên cứu &amp; Bổ sung 4 bài báo y văn mới:
+- Hackett et al. (ACL 2025 Workshop LLMSEC): Bypassing LLM Guardrails &amp; Evasion Attacks (Emoji/Unicode).
+- Jacob et al. (ACM CCS 2024): PromptShield &amp; Deployable Detection trong Low-FPR Regime (FPR &lt;= 1%).
+- Liu et al. (IEEE S&amp;P 2025): DataSentinel &amp; Game-Theoretic Minimax Detection.
+- Li &amp; Liu (ACL 2025): InjecGuard / PIGuard Mitigating Over-defense (NotInject 339 mẫu).
+- Đảm bảo 100% Open-Access PDF, xác thực metadata và cập nhật vào REFERENCES_LOG.md.</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr">
@@ -1359,8 +1458,8 @@
   <mergeCells count="7">
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="A2:U2"/>
+    <mergeCell ref="C4:F4"/>
     <mergeCell ref="A4:A5"/>
-    <mergeCell ref="C4:F4"/>
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="G4:U4"/>
     <mergeCell ref="A3:U3"/>
@@ -1710,12 +1809,12 @@
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>Soạn thảo 3 Câu hỏi nghiên cứu IEEE (RQ1-RQ3), 3 Gaps &amp; 4 Đóng góp mới</t>
+          <t>Nghiên cứu &amp; bổ sung 4 bài báo y văn mới (Hackett 2025, Jacob CCS 2024, Liu S&amp;P 2025, Li ACL 2025) vào REFERENCES_LOG.md; Soạn thảo RQ1-RQ3</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>Đang thực hiện</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
@@ -1725,7 +1824,7 @@
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>workspaces/phuongddd/</t>
+          <t>workspaces/phuongddd/References/ &amp; REFERENCES_LOG.md</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
@@ -2346,7 +2445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2527,6 +2626,88 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Meet 04</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Trực tiếp tại Campus ĐH FPT</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>4 SV (Trường, Đức, Việt, Phương) &amp; GVHD Thầy Trần Văn Ninh</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>Báo cáo slide tiến độ PI-GUARD-Present-109.pptx trực tiếp với GVHD. Tiếp thu 4 yêu cầu học thuật: định nghĩa rạch ròi Prompt Injection vs Jailbreak, phương thức tấn công &amp; hoạt động 2 mô hình (TF-IDF và DeBERTa-v3), kiểm chứng thực nghiệm mô hình/dataset y văn, và kế hoạch chạy thực nghiệm bắt buộc trước Meeting 5.</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Cả 4 thành viên cùng chuẩn bị báo cáo và slide thuyết trình; Trường &amp; Đức hoàn thiện slide; Việt &amp; Phương rà soát.
+Đầu ra: Meeting 4_10_09_26.md &amp; PI-GUARD-Present-109.pptx.</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Hoàn thành (100%)
+Final-Report/Meeting/Meeting 4_10_09_26.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>Meet 05</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>19/09/2026</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>Trực tuyến qua Google Meet với GVHD</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>4 SV (Trường, Đức, Việt, Phương) &amp; GVHD Thầy Trần Văn Ninh</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>Báo cáo kỹ thuật tiến độ 4 nhiệm vụ Meeting 5. Nhóm thẳng thắn giải trình chưa hoàn thành chọn mô hình Tầng 1 và cơ chế kết hợp 2 mô hình. GVHD góp ý tìm hiểu cơ chế chia tầng, cách thức mô hình phân tích block/ký tự/chuỗi ký tự, xử lý quá tải 200k ký tự (PDF/Ebook), prompt giấu ở cuối, và làm rõ Tier 1/2 làm gì, dùng bộ tool gì.</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>Tiến trình phân công khi tới báo cáo Meeting 5:
+- Đức: Nghiên cứu Task 1 &amp; 2 (phân biệt các key đồ án, cách thức tấn công 2 kênh Direct/Indirect).
+- Phương: Thêm 4 bài báo nghiên cứu mới vào kho y văn trong git commit (Hackett 2025, Jacob CCS 2024, Liu S&amp;P 2025, Li ACL 2025), kiểm định Open-Access PDF và cập nhật REFERENCES_LOG.md.
+- Việt: Tìm hiểu cơ chế mô hình loại bỏ encoding.
+- Trường: Thực hiện Task 3 trong truongnv (chạy 5 mô hình public nguyên bản).
+Đầu ra: Meeting 5_19_09_26.md &amp; tasks_for_meeting_5/</t>
+        </is>
+      </c>
+      <c r="G9" s="18" t="inlineStr">
+        <is>
+          <t>Hoàn thành (100%)
+Final-Report/Meeting/Meeting 5_19_09_26.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
feat(truongnv): update meeting 6 benchmarks, architectural figures, slide deck and process report
</commit_message>
<xml_diff>
--- a/Final-Report/reports/PI_GUARD_PROCESS_REPORT.xlsx
+++ b/Final-Report/reports/PI_GUARD_PROCESS_REPORT.xlsx
@@ -2445,7 +2445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2708,6 +2708,45 @@
         </is>
       </c>
     </row>
+    <row r="10" ht="95" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Meet 06</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Trực tuyến qua Google Meet với GVHD</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>4 SV (Trường, Đức, Việt, Phương) &amp; GVHD Thầy Trần Văn Ninh</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>Báo cáo kỹ thuật Meeting 6: Hoàn tất 4 yêu cầu của GVHD (Cơ chế 3 tầng, quá tải 200k ký tự, Head-Tail Priority Scanning tăng tốc 111x, toolset). Công bố quyết định đóng băng mô hình quán quân Two-Tier Cascade (v2.2-champion) và đối chuẩn 12 mô hình public.</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>Trường chủ trì thiết kế và đóng băng Two-Tier Cascade (Tier 0 Scrubber, Tier 1 TF-IDF, Tri-state Router, Tier 2 DeBERTa-v3), chạy benchmark 12 mô hình; Các thành viên cùng chạy kiểm chứng thực nghiệm.
+Đầu ra: tasks_for_meeting_6/ &amp; PI-GUARD-Present-Meeting-6.pptx</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>Hoàn thành (100%)
+Final-Report/Meeting/Meeting 6_24_09_26.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
feat: update meeting 6 reports, review 1 preparation, and member benchmark metrics
</commit_message>
<xml_diff>
--- a/Final-Report/reports/PI_GUARD_PROCESS_REPORT.xlsx
+++ b/Final-Report/reports/PI_GUARD_PROCESS_REPORT.xlsx
@@ -112,7 +112,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -134,102 +134,11 @@
         <color rgb="00B0C4DE"/>
       </bottom>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00B0C4DE"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00B0C4DE"/>
-      </left>
-      <right style="thin">
-        <color rgb="00B0C4DE"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00B0C4DE"/>
-      </left>
-      <right style="thin">
-        <color rgb="00B0C4DE"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="00B0C4DE"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00B0C4DE"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00B0C4DE"/>
-      </right>
-      <top style="thin">
-        <color rgb="00B0C4DE"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00B0C4DE"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00B0C4DE"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00B0C4DE"/>
-      </right>
-      <top style="thin">
-        <color rgb="00B0C4DE"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00B0C4DE"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D3D3D3"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D3D3D3"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D3D3D3"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D3D3D3"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -272,12 +181,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -707,32 +610,32 @@
           <t>Phân công nhiệm vụ cốt lõi</t>
         </is>
       </c>
-      <c r="D4" s="15" t="n"/>
-      <c r="E4" s="15" t="n"/>
-      <c r="F4" s="16" t="n"/>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="4" t="n"/>
       <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Tiến độ thực hiện hàng tuần (Tuần 1: 07/09/2026 – Tuần 15: 20/12/2026)</t>
         </is>
       </c>
-      <c r="H4" s="15" t="n"/>
-      <c r="I4" s="15" t="n"/>
-      <c r="J4" s="15" t="n"/>
-      <c r="K4" s="15" t="n"/>
-      <c r="L4" s="15" t="n"/>
-      <c r="M4" s="15" t="n"/>
-      <c r="N4" s="15" t="n"/>
-      <c r="O4" s="15" t="n"/>
-      <c r="P4" s="15" t="n"/>
-      <c r="Q4" s="15" t="n"/>
-      <c r="R4" s="15" t="n"/>
-      <c r="S4" s="15" t="n"/>
-      <c r="T4" s="15" t="n"/>
-      <c r="U4" s="16" t="n"/>
+      <c r="H4" s="4" t="n"/>
+      <c r="I4" s="4" t="n"/>
+      <c r="J4" s="4" t="n"/>
+      <c r="K4" s="4" t="n"/>
+      <c r="L4" s="4" t="n"/>
+      <c r="M4" s="4" t="n"/>
+      <c r="N4" s="4" t="n"/>
+      <c r="O4" s="4" t="n"/>
+      <c r="P4" s="4" t="n"/>
+      <c r="Q4" s="4" t="n"/>
+      <c r="R4" s="4" t="n"/>
+      <c r="S4" s="4" t="n"/>
+      <c r="T4" s="4" t="n"/>
+      <c r="U4" s="4" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="17" t="n"/>
-      <c r="B5" s="17" t="n"/>
+      <c r="A5" s="5" t="n"/>
+      <c r="B5" s="5" t="n"/>
       <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Nhiệm vụ 1</t>
@@ -885,26 +788,26 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Thực hiện Task 3 (Replication Lab):
-- Tải và chạy thực nghiệm 5 mô hình y văn public nguyên bản trong truongnv: PIGuard DeBERTa-v3, Ayub MiniLM, Meta Prompt-Guard, Jain Perplexity, InstructDetector.
-- Đo đạc trên 5 benchmark mở (NotInject, WildGuard, BIPIA).
-- Đối soát số liệu đo đạc khớp bài báo ACL 2025.</t>
+          <t>Bối cảnh &amp; Phân loại:
+- Soạn thảo Chapter 1 (Introduction).
+- Phân loại Threat Taxonomy (OWASP).
+- Lỗ hổng Von Neumann NLP.</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>Literature Review:
-- Soạn thảo Chapter 2 (Literature Review).
-- Khảo sát SOTA Guardrails.
-- Dàn ý slide 9 trang Review 1.</t>
+          <t>Báo cáo Meeting 6 (26/09) &amp; Docs:
+- Hoàn thiện toàn văn Report No.1 (Chapter 1) &amp; Report No.2 (Chapter 2).
+- Cùng Đức trực tiếp tạo bộ slide báo cáo tiến độ Meeting 6 (SLIDE_DECK_MEETING_6.md).
+- Ngày 26/09: Báo cáo trực tiếp tại trường với GVHD ThS. Trần Văn Ninh; cùng Phương thuyết trình Phần 4 (Đề xuất kiến trúc Two-Tier Cascade của đồ án).</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>BẢO VỆ REVIEW 1 (GVHD):
-- Hoàn thiện Report No.1 &amp; No.2.
-- Thiết kế Slide PPTX &amp; tập diễn tập.
-- Bảo vệ thành công Review 1.</t>
+          <t>BẢO VỆ REVIEW 1 (THỨ 4: 30/09/2026):
+- Tóm gọn toàn bộ nội dung báo cáo ngày 26/09 thành hồ sơ nghiệm thu chính thức Review 1.
+- Đóng gói toàn văn Report No.1 (Chapter 1) &amp; Report No.2 (Chapter 2) nộp cho GVHD.
+- Điều phối diễn tập thuyết trình 15 phút và bảo vệ thành công mốc Review 1.</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
@@ -1037,26 +940,25 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>Nghiên cứu Task 1 &amp; 2 (Keys &amp; Attack Vectors):
-- Phân biệt 2 key đồ án: Prompt Injection vs. Jailbreak.
-- Phân tích cách thức hoạt động &amp; bề mặt tấn công 2 kênh: Direct Chat vs. Indirect File/RAG.
-- Khung 5 trục NIST AI 100-2e2025, luồng thực thi và blast radius.</t>
+          <t>Threat Model &amp; Attack Surface:
+- Xây dựng sơ đồ NIST AI 100-2e2025.
+- Khóa chặt Attack Surface /v1/chat.
+- Thiết kế kiến trúc bảo vệ 3 lớp.</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>Chuẩn bị Review 1:
-- Chuẩn bị slide Threat Model &amp; 3L.
-- Xây dựng script baseline TF-IDF mẫu.
-- Thử nghiệm feature extraction.</t>
+          <t>Slide &amp; Thuyết trình Meeting 6 (26/09):
+- Cùng Trường trực tiếp thiết kế cấu trúc và hoàn thiện bộ slide báo cáo tiến độ Meeting 6.
+- Ngày 26/09: Báo cáo trực tiếp tại trường với GVHD ThS. Trần Văn Ninh; thuyết trình Phần 1 (Lỗ hổng ranh giới phẳng &amp; phân loại tấn công) và Phần 2 (Cơ sở lý thuyết, SOTA, Guardrail Trilemma).</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>BẢO VỆ REVIEW 1 (GVHD):
-- Trình bày Threat Model &amp; Kiến trúc 3L.
-- Phản biện phương pháp luận baseline.
-- Hoàn thành mốc Review 1.</t>
+          <t>BẢO VỆ REVIEW 1 (THỨ 4: 30/09/2026):
+- Cùng Phương tóm gọn nội dung báo cáo ngày 26/09 và hoàn thiện bộ Slide thuyết trình 15 phút Review 1.
+- Phụ trách thuyết trình Phần 1 &amp; Phần 2 trong buổi bảo vệ Review 1 trước GVHD.
+- Nghiệm thu thành công cột mốc Review 1.</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
@@ -1189,26 +1091,25 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>Tìm hiểu cơ chế loại bỏ Encoding:
-- Khảo sát các kỹ thuật mã hóa né tránh: Base64, Hexadecimal, Leetspeak, Rot13, ciphers.
-- Tìm hiểu cơ chế bóc tách chuỗi và chuẩn hóa (Tier-0 Scrubber).
-- Đánh giá ảnh hưởng của encoding làm mù tokenizer mô hình.</t>
+          <t>Khảo sát Y văn Guardrail:
+- Đối sánh các trường phái Guardrail.
+- Khảo sát các dòng Target LLMs.
+- Soạn thảo luận giải chọn mô hình.</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>Kịch bản Minh họa Đề bài:
-- Thiết kế ma trận 4 Kịch bản Demo 2x2.
-- Xây dựng luồng tấn công vs đề xuất bảo vệ.
-- Chuẩn bị slide thuyết trình Review 1.</t>
+          <t>Thực nghiệm &amp; Báo cáo Meeting 6 (26/09):
+- Chạy thực nghiệm đo đạc độc lập 6 mô hình y văn trên bộ benchmark cross-dataset D1–D6 trong sandbox.
+- Ngày 26/09: Báo cáo trực tiếp tại trường với GVHD ThS. Trần Văn Ninh; thuyết trình Phần 3 (Kết quả thực nghiệm đối chuẩn chéo D1–D6 chỉ ra các failure modes y văn).</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>BẢO VỆ REVIEW 1 (GVHD):
-- Trình bày Luận giải mô hình &amp; Demo đề bài.
-- Báo cáo cơ sở khoa học DeBERTa-v3.
-- Hoàn thành mốc Review 1.</t>
+          <t>BẢO VỆ REVIEW 1 (THỨ 4: 30/09/2026):
+- Tóm gọn số liệu thực nghiệm D1–D6 vào Mục 2.3 (Research Gaps) của Report No.2.
+- Phụ trách báo cáo phần thực nghiệm đối chuẩn (Phần 3) trong buổi bảo vệ Review 1 trước GVHD.
+- Nghiệm thu thành công cột mốc Review 1.</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
@@ -1341,28 +1242,26 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>Nghiên cứu &amp; Bổ sung 4 bài báo y văn mới:
-- Hackett et al. (ACL 2025 Workshop LLMSEC): Bypassing LLM Guardrails &amp; Evasion Attacks (Emoji/Unicode).
-- Jacob et al. (ACM CCS 2024): PromptShield &amp; Deployable Detection trong Low-FPR Regime (FPR &lt;= 1%).
-- Liu et al. (IEEE S&amp;P 2025): DataSentinel &amp; Game-Theoretic Minimax Detection.
-- Li &amp; Liu (ACL 2025): InjecGuard / PIGuard Mitigating Over-defense (NotInject 339 mẫu).
-- Đảm bảo 100% Open-Access PDF, xác thực metadata và cập nhật vào REFERENCES_LOG.md.</t>
+          <t>Research Questions &amp; Gaps:
+- Soạn thảo 3 Câu hỏi IEEE (RQ1-RQ3).
+- Xác định 3 Gaps &amp; 4 Đóng góp mới.
+- Định vị ranh giới In-scope/Out-of-scope.</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>Slide Outline Review 1:
-- Thiết kế bộ slide 9 trang Review 1.
-- Dựng demo UI mô phỏng 4 kịch bản.
-- Soạn kịch bản thuyết trình 15 phút.</t>
+          <t>Đề xuất Mô hình &amp; Báo cáo Meeting 6 (26/09):
+- Phân tích giải pháp xử lý văn bản dài 200k ký tự và chống prompt giấu ở đuôi (Head-and-Tail Priority Scanning).
+- Ngày 26/09: Báo cáo trực tiếp tại trường với GVHD ThS. Trần Văn Ninh; cùng Trường thuyết trình Phần 4 (Đề xuất kiến trúc Two-Tier Cascade của đồ án).
+- Hỗ trợ rà soát docs Chapter 1 &amp; 2.</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>BẢO VỆ REVIEW 1 (GVHD):
-- Trình bày RQ1-RQ3 &amp; Đóng góp mới.
-- Điều phối trình chiếu slide Review 1.
-- Hoàn thành mốc Review 1.</t>
+          <t>BẢO VỆ REVIEW 1 (THỨ 4: 30/09/2026):
+- Cùng Đức hoàn thiện bộ slide PowerPoint 15 phút Review 1 theo chuẩn ĐH FPT.
+- Cùng Trường phụ trách thuyết trình phần đề xuất kiến trúc (Phần 4) tại Review 1.
+- Nghiệm thu thành công cột mốc Review 1.</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">
@@ -1458,8 +1357,8 @@
   <mergeCells count="7">
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="A2:U2"/>
+    <mergeCell ref="A4:A5"/>
     <mergeCell ref="C4:F4"/>
-    <mergeCell ref="A4:A5"/>
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="G4:U4"/>
     <mergeCell ref="A3:U3"/>
@@ -1664,9 +1563,9 @@
           <t>Soạn thảo Chapter 1: Background &amp; Problem Statement (Lỗ hổng Von Neumann NLP)</t>
         </is>
       </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
@@ -1701,9 +1600,9 @@
           <t>Phân loại Threat Taxonomy (Direct/Indirect Injection vs Jailbreak theo OWASP)</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">
@@ -1738,9 +1637,9 @@
           <t>Xây dựng Threat Model (NIST AI 100-2e2025) &amp; Attack Surface (/v1/chat)</t>
         </is>
       </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
@@ -1775,9 +1674,9 @@
           <t>Thiết kế Kiến trúc bảo vệ 3 lớp &amp; Cơ chế phòng thủ độ bền Robustness</t>
         </is>
       </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
@@ -1809,10 +1708,10 @@
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>Nghiên cứu &amp; bổ sung 4 bài báo y văn mới (Hackett 2025, Jacob CCS 2024, Liu S&amp;P 2025, Li ACL 2025) vào REFERENCES_LOG.md; Soạn thảo RQ1-RQ3</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
+          <t>Soạn thảo 3 Câu hỏi nghiên cứu IEEE (RQ1-RQ3), 3 Gaps &amp; 4 Đóng góp mới</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>Hoàn thành</t>
         </is>
@@ -1824,7 +1723,7 @@
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>workspaces/phuongddd/References/ &amp; REFERENCES_LOG.md</t>
+          <t>workspaces/phuongddd/</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
@@ -1849,9 +1748,9 @@
           <t>Khảo sát SOTA Guardrails, Luận giải chọn mô hình &amp; Khảo sát 5 Target LLMs</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="E13" s="10" t="inlineStr">
@@ -1886,9 +1785,9 @@
           <t>Thiết kế Ma trận 4 Kịch bản Minh họa Đề bài (2x2: Vulnerable vs Proposed Protected)</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr">
@@ -1923,9 +1822,9 @@
           <t>Hoàn thiện toàn văn Report No.1: Introduction (Chapter 1 — 10% Process Mark)</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr">
@@ -1960,9 +1859,9 @@
           <t>Hoàn thiện toàn văn Report No.2: Literature Review (Chapter 2 — 25% Process Mark)</t>
         </is>
       </c>
-      <c r="D16" s="12" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">
@@ -1994,27 +1893,27 @@
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>Thiết kế dàn ý slide 9 trang Review 1 Presentation Slides (Bao gồm 2 Chương)</t>
-        </is>
-      </c>
-      <c r="D17" s="12" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
+          <t>Báo cáo Meeting 6 trực tiếp tại trường với GVHD (26/09): Trường &amp; Đức làm slide; Đức thuyết trình P1-P2; Việt P3; Trường &amp; Phương P4</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>Phương</t>
+          <t>Cả 4 thành viên</t>
         </is>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>workspaces/truongnv/docs/</t>
+          <t>Final-Report/Meeting/Meeting 6_26_09_26.md</t>
         </is>
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>27/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
     </row>
@@ -2031,12 +1930,12 @@
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>Thiết kế slide PowerPoint (.pptx) &amp; Tập dượt thuyết trình 15 phút (2 Chương)</t>
-        </is>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
-        <is>
-          <t>Chưa bắt đầu</t>
+          <t>Tóm gọn toàn bộ báo cáo ngày 26/9 thành hồ sơ Review 1 &amp; Hoàn thiện slide PPTX 15 phút</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>Đang thực hiện</t>
         </is>
       </c>
       <c r="E18" s="10" t="inlineStr">
@@ -2051,7 +1950,7 @@
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
     </row>
@@ -2071,9 +1970,9 @@
           <t>Họp tổng kết tuần, cập nhật Process Report Excel &amp; Nộp Report 1 &amp; 2 cho GVHD</t>
         </is>
       </c>
-      <c r="D19" s="13" t="inlineStr">
-        <is>
-          <t>Chưa bắt đầu</t>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>Đang thực hiện</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">
@@ -2105,12 +2004,12 @@
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>CỘT MỐC 1 — BẢO VỆ REVIEW 1 TRƯỚC GVHD (CHAPTERS 1 &amp; 2)</t>
-        </is>
-      </c>
-      <c r="D20" s="13" t="inlineStr">
-        <is>
-          <t>Chưa bắt đầu</t>
+          <t>CỘT MỐC 1 — BẢO VỆ REVIEW 1 TRƯỚC GVHD (CHAPTERS 1 &amp; 2 - THỨ 4: 30/09/2026)</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Đang thực hiện</t>
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr">
@@ -2125,7 +2024,7 @@
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>04/10/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
     </row>
@@ -2543,7 +2442,7 @@
       <c r="G5" s="14" t="inlineStr">
         <is>
           <t>Hoàn thành (100%)
-reports/Meeting/Meeting 1_29_08_26.md</t>
+Final-Report/Meeting/Meeting 1_29_08_26.md</t>
         </is>
       </c>
     </row>
@@ -2582,7 +2481,7 @@
       <c r="G6" s="14" t="inlineStr">
         <is>
           <t>Hoàn thành (100%)
-reports/Meeting/Meeting 2_01_09_26.md</t>
+Final-Report/Meeting/Meeting 2_01_09_26.md</t>
         </is>
       </c>
     </row>
@@ -2626,89 +2525,85 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="18" t="inlineStr">
+    <row r="8" ht="80" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Meet 04</t>
         </is>
       </c>
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>10/09/2026</t>
         </is>
       </c>
-      <c r="C8" s="18" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Trực tiếp tại Campus ĐH FPT</t>
         </is>
       </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>4 SV (Trường, Đức, Việt, Phương) &amp; GVHD Thầy Trần Văn Ninh</t>
-        </is>
-      </c>
-      <c r="E8" s="18" t="inlineStr">
-        <is>
-          <t>Báo cáo slide tiến độ PI-GUARD-Present-109.pptx trực tiếp với GVHD. Tiếp thu 4 yêu cầu học thuật: định nghĩa rạch ròi Prompt Injection vs Jailbreak, phương thức tấn công &amp; hoạt động 2 mô hình (TF-IDF và DeBERTa-v3), kiểm chứng thực nghiệm mô hình/dataset y văn, và kế hoạch chạy thực nghiệm bắt buộc trước Meeting 5.</t>
-        </is>
-      </c>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>Cả 4 thành viên cùng chuẩn bị báo cáo và slide thuyết trình; Trường &amp; Đức hoàn thiện slide; Việt &amp; Phương rà soát.
-Đầu ra: Meeting 4_10_09_26.md &amp; PI-GUARD-Present-109.pptx.</t>
-        </is>
-      </c>
-      <c r="G8" s="18" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>4 SV (Trường, Đức, Việt, Phương) &amp; GVHD</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>Báo cáo trực tiếp tại trường: Thuyết trình bộ slide tiến độ PI-GUARD-Present-109.pptx; tiếp thu 4 yêu cầu học thuật &amp; kỹ thuật trọng tâm từ GVHD (phân biệt rạch ròi Prompt Injection vs Jailbreak, phương thức tấn công 2 kênh Ingress, kiểm chứng thực nghiệm mã nguồn y văn và công thức tinh chỉnh đồ án).</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>Trường điều phối; cả 4 thành viên trực tiếp chạy độc lập toàn bộ pipeline thực nghiệm trên máy cá nhân để nắm chắc số liệu.
+Đầu ra: Meeting 4_10_09_26.md.</t>
+        </is>
+      </c>
+      <c r="G8" s="14" t="inlineStr">
         <is>
           <t>Hoàn thành (100%)
 Final-Report/Meeting/Meeting 4_10_09_26.md</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+    <row r="9" ht="80" customHeight="1">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Meet 05</t>
         </is>
       </c>
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>19/09/2026</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>Trực tuyến qua Google Meet với GVHD</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>4 SV (Trường, Đức, Việt, Phương) &amp; GVHD Thầy Trần Văn Ninh</t>
-        </is>
-      </c>
-      <c r="E9" s="18" t="inlineStr">
-        <is>
-          <t>Báo cáo kỹ thuật tiến độ 4 nhiệm vụ Meeting 5. Nhóm thẳng thắn giải trình chưa hoàn thành chọn mô hình Tầng 1 và cơ chế kết hợp 2 mô hình. GVHD góp ý tìm hiểu cơ chế chia tầng, cách thức mô hình phân tích block/ký tự/chuỗi ký tự, xử lý quá tải 200k ký tự (PDF/Ebook), prompt giấu ở cuối, và làm rõ Tier 1/2 làm gì, dùng bộ tool gì.</t>
-        </is>
-      </c>
-      <c r="F9" s="18" t="inlineStr">
-        <is>
-          <t>Tiến trình phân công khi tới báo cáo Meeting 5:
-- Đức: Nghiên cứu Task 1 &amp; 2 (phân biệt các key đồ án, cách thức tấn công 2 kênh Direct/Indirect).
-- Phương: Thêm 4 bài báo nghiên cứu mới vào kho y văn trong git commit (Hackett 2025, Jacob CCS 2024, Liu S&amp;P 2025, Li ACL 2025), kiểm định Open-Access PDF và cập nhật REFERENCES_LOG.md.
-- Việt: Tìm hiểu cơ chế mô hình loại bỏ encoding.
-- Trường: Thực hiện Task 3 trong truongnv (chạy 5 mô hình public nguyên bản).
-Đầu ra: Meeting 5_19_09_26.md &amp; tasks_for_meeting_5/</t>
-        </is>
-      </c>
-      <c r="G9" s="18" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Trực tuyến (Google Meet với GVHD)</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>4 SV (Trường, Đức, Việt, Phương) &amp; GVHD</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>Báo cáo kỹ thuật trực tuyến: Thẳng thắn giải trình tình trạng chưa hoàn thành task chọn mô hình Tầng 1 và cơ chế kết hợp; tiếp thu chỉ đạo về bóc tách chuỗi/block, giải quyết quá tải 200k ký tự, chống prompt giấu ở cuối, và làm rõ Tier 1/Tier 2 làm gì, dùng toolset gì.</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>Cả nhóm cùng tìm hiểu cơ chế băm khối Sliding Window và thuật toán Head &amp; Tail Scan.
+Đầu ra: Meeting 5_19_09_26.md.</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
         <is>
           <t>Hoàn thành (100%)
 Final-Report/Meeting/Meeting 5_19_09_26.md</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="95" customHeight="1">
+    <row r="10" ht="80" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Meet 06</t>
@@ -2716,34 +2611,34 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>Trực tuyến qua Google Meet với GVHD</t>
+          <t>Trực tiếp tại Campus ĐH FPT</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>4 SV (Trường, Đức, Việt, Phương) &amp; GVHD Thầy Trần Văn Ninh</t>
+          <t>4 SV (Trường, Đức, Việt, Phương) &amp; GVHD</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
         <is>
-          <t>Báo cáo kỹ thuật Meeting 6: Hoàn tất 4 yêu cầu của GVHD (Cơ chế 3 tầng, quá tải 200k ký tự, Head-Tail Priority Scanning tăng tốc 111x, toolset). Công bố quyết định đóng băng mô hình quán quân Two-Tier Cascade (v2.2-champion) và đối chuẩn 12 mô hình public.</t>
+          <t>Báo cáo kỹ thuật trực tiếp tại trường: Giải quyết triệt để 4 gợi mở từ Meeting 5. Trường &amp; Đức làm slide; Đức thuyết trình P1-P2 (Lý thuyết, SOTA, Trilemma); Việt báo cáo P3 (Thực nghiệm D1–D6); Trường &amp; Phương báo cáo P4 (Đề xuất kiến trúc Two-Tier Cascade). GVHD đánh giá cao tiến bộ vượt bậc.</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>Trường chủ trì thiết kế và đóng băng Two-Tier Cascade (Tier 0 Scrubber, Tier 1 TF-IDF, Tri-state Router, Tier 2 DeBERTa-v3), chạy benchmark 12 mô hình; Các thành viên cùng chạy kiểm chứng thực nghiệm.
-Đầu ra: tasks_for_meeting_6/ &amp; PI-GUARD-Present-Meeting-6.pptx</t>
+          <t>Tóm gọn toàn bộ báo cáo ngày 26/09 để chuẩn bị hồ sơ bảo vệ Review 1 vào Thứ 4 tuần sau (30/09/2026).
+Đầu ra: Meeting 6_26_09_26.md &amp; SLIDE_DECK_MEETING_6.md.</t>
         </is>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
           <t>Hoàn thành (100%)
-Final-Report/Meeting/Meeting 6_24_09_26.md</t>
+Final-Report/Meeting/Meeting 6_26_09_26.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: add repo timeline and enforce publication boundary
</commit_message>
<xml_diff>
--- a/Final-Report/reports/PI_GUARD_PROCESS_REPORT.xlsx
+++ b/Final-Report/reports/PI_GUARD_PROCESS_REPORT.xlsx
@@ -817,9 +817,8 @@
         </x:is>
       </x:c>
       <x:c r="J6" s="6" t="str">
-        <x:v>REVIEW 1 HOÀN TẤT (04/10/2026, theo xác nhận của người dùng).
-- Báo cáo tổng kết Review 1: workspaces/truongnv/reports/report_for_review1/REVIEW_1_COMPLETION_REPORT_2026-10-04.md.
-- Trạng thái này không xác nhận nghiệm thu mô hình hoặc cascade.</x:v>
+        <x:v>Review 1: snapshot 03/10; hoàn tất 04/10 theo xác nhận.
+Report 1/2 đã ghi hoàn thành; chưa có chứng cứ gửi GVHD. Không phải nghiệm thu mô hình.</x:v>
       </x:c>
       <x:c r="K6" s="6" t="inlineStr">
         <x:is>
@@ -965,9 +964,8 @@
         </x:is>
       </x:c>
       <x:c r="J7" s="7" t="str">
-        <x:v>REVIEW 1 HOÀN TẤT (04/10/2026, theo xác nhận của người dùng).
-- Báo cáo tổng kết Review 1: workspaces/truongnv/reports/report_for_review1/REVIEW_1_COMPLETION_REPORT_2026-10-04.md.
-- Trạng thái này không xác nhận nghiệm thu mô hình hoặc cascade.</x:v>
+        <x:v>Review 1: snapshot 03/10; hoàn tất 04/10 theo xác nhận.
+Report 1/2 đã ghi hoàn thành; chưa có chứng cứ gửi GVHD. Không phải nghiệm thu mô hình.</x:v>
       </x:c>
       <x:c r="K7" s="7" t="inlineStr">
         <x:is>
@@ -1113,9 +1111,8 @@
         </x:is>
       </x:c>
       <x:c r="J8" s="6" t="str">
-        <x:v>REVIEW 1 HOÀN TẤT (04/10/2026, theo xác nhận của người dùng).
-- Báo cáo tổng kết Review 1: workspaces/truongnv/reports/report_for_review1/REVIEW_1_COMPLETION_REPORT_2026-10-04.md.
-- Trạng thái này không xác nhận nghiệm thu mô hình hoặc cascade.</x:v>
+        <x:v>Review 1: snapshot 03/10; hoàn tất 04/10 theo xác nhận.
+Report 1/2 đã ghi hoàn thành; chưa có chứng cứ gửi GVHD. Không phải nghiệm thu mô hình.</x:v>
       </x:c>
       <x:c r="K8" s="6" t="inlineStr">
         <x:is>
@@ -1262,9 +1259,8 @@
         </x:is>
       </x:c>
       <x:c r="J9" s="7" t="str">
-        <x:v>REVIEW 1 HOÀN TẤT (04/10/2026, theo xác nhận của người dùng).
-- Báo cáo tổng kết Review 1: workspaces/truongnv/reports/report_for_review1/REVIEW_1_COMPLETION_REPORT_2026-10-04.md.
-- Trạng thái này không xác nhận nghiệm thu mô hình hoặc cascade.</x:v>
+        <x:v>Review 1: snapshot 03/10; hoàn tất 04/10 theo xác nhận.
+Report 1/2 đã ghi hoàn thành; chưa có chứng cứ gửi GVHD. Không phải nghiệm thu mô hình.</x:v>
       </x:c>
       <x:c r="K9" s="7" t="inlineStr">
         <x:is>
@@ -1501,10 +1497,8 @@
           <x:t>Trường &amp; Đức</x:t>
         </x:is>
       </x:c>
-      <x:c r="F6" s="10" t="inlineStr">
-        <x:is>
-          <x:t>reports/PI-GUARD-Present-109.pptx</x:t>
-        </x:is>
+      <x:c r="F6" s="10" t="str">
+        <x:v>Final-Report/Meeting/Meeting 3_08_09_26.md</x:v>
       </x:c>
       <x:c r="G6" s="9" t="inlineStr">
         <x:is>
@@ -1982,15 +1976,11 @@
           <x:t>Trường (Leader)</x:t>
         </x:is>
       </x:c>
-      <x:c r="F19" s="10" t="inlineStr">
-        <x:is>
-          <x:t>PI_GUARD_PROCESS_REPORT.xlsx</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G19" s="9" t="inlineStr">
-        <x:is>
-          <x:t>03/10/2026</x:t>
-        </x:is>
+      <x:c r="F19" s="10" t="str">
+        <x:v>PI_GUARD_PROCESS_REPORT.xlsx</x:v>
+      </x:c>
+      <x:c r="G19" s="9" t="str">
+        <x:v>03/10/2026</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="60" customHeight="1">
@@ -2035,10 +2025,8 @@
           <x:t>Tuần 5 - 6 (05/10 - 18/10)</x:t>
         </x:is>
       </x:c>
-      <x:c r="C21" s="10" t="inlineStr">
-        <x:is>
-          <x:t>Thu thập Dataset đa nguồn, Group-Aware Split &amp; Huấn luyện Baseline ML</x:t>
-        </x:is>
+      <x:c r="C21" s="10" t="str">
+        <x:v>Duyệt nguồn/nhãn; group-aware split; fit baseline TF-IDF ba lớp</x:v>
       </x:c>
       <x:c r="D21" s="13" t="inlineStr">
         <x:is>
@@ -2050,10 +2038,8 @@
           <x:t>Trường &amp; Đức</x:t>
         </x:is>
       </x:c>
-      <x:c r="F21" s="10" t="inlineStr">
-        <x:is>
-          <x:t>data/processed/ &amp; models/baseline/</x:t>
-        </x:is>
+      <x:c r="F21" s="10" t="str">
+        <x:v>L2 model + metrics</x:v>
       </x:c>
       <x:c r="G21" s="9" t="inlineStr">
         <x:is>
@@ -2072,10 +2058,8 @@
           <x:t>Tuần 7 (19/10 - 25/10)</x:t>
         </x:is>
       </x:c>
-      <x:c r="C22" s="10" t="inlineStr">
-        <x:is>
-          <x:t>Soạn thảo, cập nhật docs Chapter 3 (Methodology - Report No.3) &amp; Chuẩn bị Slide Review 2</x:t>
-        </x:is>
+      <x:c r="C22" s="10" t="str">
+        <x:v>Fine-tune DeBERTa; tích hợp demo L2/L3; soạn Chapter 3 và slide</x:v>
       </x:c>
       <x:c r="D22" s="13" t="inlineStr">
         <x:is>
@@ -2087,10 +2071,8 @@
           <x:t>Đức &amp; Trường</x:t>
         </x:is>
       </x:c>
-      <x:c r="F22" s="10" t="inlineStr">
-        <x:is>
-          <x:t>docs/thesis/chapters/03_Methodology.md &amp; Slide Review 2</x:t>
-        </x:is>
+      <x:c r="F22" s="10" t="str">
+        <x:v>Checkpoint; inference thật; tài liệu Review 2</x:v>
       </x:c>
       <x:c r="G22" s="9" t="inlineStr">
         <x:is>
@@ -2109,10 +2091,8 @@
           <x:t>Tuần 8 (26/10 - 01/11)</x:t>
         </x:is>
       </x:c>
-      <x:c r="C23" s="10" t="inlineStr">
-        <x:is>
-          <x:t>CỘT MỐC 2 — BẢO VỆ REVIEW 2 TRƯỚC GVHD (CHAPTER 3), Nộp Report No.3 &amp; Cập nhật Docs hoàn chỉnh</x:t>
-        </x:is>
+      <x:c r="C23" s="10" t="str">
+        <x:v>Review 2: Chapter 3 và demo model PI-Guard ba nhãn</x:v>
       </x:c>
       <x:c r="D23" s="13" t="inlineStr">
         <x:is>
@@ -2124,10 +2104,8 @@
           <x:t>Cả 4 thành viên</x:t>
         </x:is>
       </x:c>
-      <x:c r="F23" s="10" t="inlineStr">
-        <x:is>
-          <x:t>Biên bản nghiệm thu Review 2 &amp; Chapter 3 final</x:t>
-        </x:is>
+      <x:c r="F23" s="10" t="str">
+        <x:v>Demo thật, provenance và checklist trạng thái</x:v>
       </x:c>
       <x:c r="G23" s="9" t="inlineStr">
         <x:is>
@@ -2146,10 +2124,8 @@
           <x:t>Tuần 9 - 10 (02/11 - 15/11)</x:t>
         </x:is>
       </x:c>
-      <x:c r="C24" s="10" t="inlineStr">
-        <x:is>
-          <x:t>Fine-tuning DeBERTa-v3, Đánh giá Adversarial Robustness &amp; Nộp Report No.4</x:t>
-        </x:is>
+      <x:c r="C24" s="10" t="str">
+        <x:v>Đánh giá robustness DeBERTa; hoàn tất Report No.4</x:v>
       </x:c>
       <x:c r="D24" s="13" t="inlineStr">
         <x:is>
@@ -2161,10 +2137,8 @@
           <x:t>Việt &amp; Đức</x:t>
         </x:is>
       </x:c>
-      <x:c r="F24" s="10" t="inlineStr">
-        <x:is>
-          <x:t>Report No.4 &amp; models/</x:t>
-        </x:is>
+      <x:c r="F24" s="10" t="str">
+        <x:v>Report No.4; metrics từng lớp; checkpoint/hash</x:v>
       </x:c>
       <x:c r="G24" s="9" t="inlineStr">
         <x:is>
@@ -2507,18 +2481,13 @@
           <x:t>Đánh giá kết quả nghiên cứu và thống nhất slide báo cáo tiến độ gặp GVHD ngày 10/09/2026.</x:t>
         </x:is>
       </x:c>
-      <x:c r="F7" s="10" t="inlineStr">
-        <x:is>
-          <x:t>Trường và Đức trực tiếp tạo slide, biên soạn nội dung và hoàn thiện toàn bộ bộ Slide 22 trang (PI-GUARD-Present-109.pptx); Việt và Phương rà soát, thống nhất hoàn toàn và không có ý kiến bổ sung.
-Đầu ra: Meeting 3_08_09_26.md &amp; Final-Report/PI-GUARD-Present-109.pptx.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G7" s="14" t="inlineStr">
-        <x:is>
-          <x:t>Hoàn thành (100%)
-Final-Report/Meeting/Meeting 3_08_09_26.md
-Final-Report/PI-GUARD-Present-109.pptx</x:t>
-        </x:is>
+      <x:c r="F7" s="10" t="str">
+        <x:v>Trường và Đức hoàn thiện bộ slide 22 trang; Việt và Phương rà soát, không có ý kiến bổ sung.
+Đầu ra: Meeting 3_08_09_26.md; slide đã gỡ ngày 08/10/2026.</x:v>
+      </x:c>
+      <x:c r="G7" s="14" t="str">
+        <x:v>Hoàn thành (100%)
+Final-Report/Meeting/Meeting 3_08_09_26.md</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="80" customHeight="1">

</xml_diff>

<commit_message>
chore: publish single-maintainer updates and consolidate experiment reports
</commit_message>
<xml_diff>
--- a/Final-Report/reports/PI_GUARD_PROCESS_REPORT.xlsx
+++ b/Final-Report/reports/PI_GUARD_PROCESS_REPORT.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:workbookPr/>
   <x:workbookProtection/>
   <x:bookViews>
@@ -74,10 +74,10 @@
       <x:sz val="10"/>
     </x:font>
     <x:font>
-      <x:b/>
+      <x:name val="Calibri"/>
+      <x:b val="1"/>
+      <x:color rgb="FF375623"/>
       <x:sz val="10"/>
-      <x:color rgb="FF375623"/>
-      <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
   <x:fills count="8">
@@ -123,7 +123,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="9">
     <x:border>
       <x:left/>
       <x:right/>
@@ -145,11 +145,88 @@
         <x:color rgb="00B0C4DE"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="00B0C4DE"/>
+      </x:left>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="00B0C4DE"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="00B0C4DE"/>
+      </x:right>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="00B0C4DE"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="00B0C4DE"/>
+      </x:right>
+      <x:top/>
+      <x:bottom style="thin">
+        <x:color rgb="00B0C4DE"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="00B0C4DE"/>
+      </x:top>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="00B0C4DE"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="00B0C4DE"/>
+      </x:top>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="00B0C4DE"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="00B0C4DE"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="00B0C4DE"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="00B0C4DE"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="00B0C4DE"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="20">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="0" pivotButton="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="0" pivotButton="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
@@ -193,8 +270,14 @@
     <x:xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" quotePrefix="0" pivotButton="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="0" quotePrefix="0" pivotButton="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" quotePrefix="0" pivotButton="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" quotePrefix="0" pivotButton="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" quotePrefix="0" pivotButton="0"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -624,32 +707,32 @@
           <x:t>Phân công nhiệm vụ cốt lõi</x:t>
         </x:is>
       </x:c>
-      <x:c r="D4" s="4" t="n"/>
-      <x:c r="E4" s="4" t="n"/>
-      <x:c r="F4" s="4" t="n"/>
+      <x:c r="D4" s="16" t="n"/>
+      <x:c r="E4" s="16" t="n"/>
+      <x:c r="F4" s="17" t="n"/>
       <x:c r="G4" s="4" t="inlineStr">
         <x:is>
           <x:t>Tiến độ thực hiện hàng tuần (Tuần 1: 07/09/2026 – Tuần 15: 20/12/2026)</x:t>
         </x:is>
       </x:c>
-      <x:c r="H4" s="4" t="n"/>
-      <x:c r="I4" s="4" t="n"/>
-      <x:c r="J4" s="4" t="n"/>
-      <x:c r="K4" s="4" t="n"/>
-      <x:c r="L4" s="4" t="n"/>
-      <x:c r="M4" s="4" t="n"/>
-      <x:c r="N4" s="4" t="n"/>
-      <x:c r="O4" s="4" t="n"/>
-      <x:c r="P4" s="4" t="n"/>
-      <x:c r="Q4" s="4" t="n"/>
-      <x:c r="R4" s="4" t="n"/>
-      <x:c r="S4" s="4" t="n"/>
-      <x:c r="T4" s="4" t="n"/>
-      <x:c r="U4" s="4" t="n"/>
+      <x:c r="H4" s="16" t="n"/>
+      <x:c r="I4" s="16" t="n"/>
+      <x:c r="J4" s="16" t="n"/>
+      <x:c r="K4" s="16" t="n"/>
+      <x:c r="L4" s="16" t="n"/>
+      <x:c r="M4" s="16" t="n"/>
+      <x:c r="N4" s="16" t="n"/>
+      <x:c r="O4" s="16" t="n"/>
+      <x:c r="P4" s="16" t="n"/>
+      <x:c r="Q4" s="16" t="n"/>
+      <x:c r="R4" s="16" t="n"/>
+      <x:c r="S4" s="16" t="n"/>
+      <x:c r="T4" s="16" t="n"/>
+      <x:c r="U4" s="17" t="n"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="5" t="n"/>
-      <x:c r="B5" s="5" t="n"/>
+      <x:c r="A5" s="18" t="n"/>
+      <x:c r="B5" s="18" t="n"/>
       <x:c r="C5" s="5" t="inlineStr">
         <x:is>
           <x:t>Nhiệm vụ 1</x:t>
@@ -761,7 +844,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="6" ht="110" customHeight="1">
+    <x:row r="6" ht="190" customHeight="1">
       <x:c r="A6" s="6" t="inlineStr">
         <x:is>
           <x:t>SE182034</x:t>
@@ -816,17 +899,16 @@
 - Ngày 26/09: Báo cáo trực tiếp tại trường với GVHD ThS. Trần Văn Ninh; cùng Phương thuyết trình Phần 4 (Đề xuất kiến trúc Two-Tier Cascade của đồ án).</x:t>
         </x:is>
       </x:c>
-      <x:c r="J6" s="6" t="str">
-        <x:v>Review 1: snapshot 03/10; hoàn tất 04/10 theo xác nhận.
-Report 1/2 đã ghi hoàn thành; chưa có chứng cứ gửi GVHD. Không phải nghiệm thu mô hình.</x:v>
-      </x:c>
-      <x:c r="K6" s="6" t="inlineStr">
-        <x:is>
-          <x:t>Data Engineering:
-- Tải 5 datasets từ Hugging Face.
-- Cài đặt Group-Aware Split.
-- Làm sạch &amp; khử trùng lặp dữ liệu.</x:t>
-        </x:is>
+      <x:c r="J6" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Review 1: snapshot 03/10; hoàn tất 04/10 theo xác nhận.
+Report 1/2 đã ghi hoàn thành; chưa có chứng cứ gửi GVHD. Không phải nghiệm thu mô hình.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K6" s="6" t="str">
+        <x:v>V7.1 L2: five fits shared the same 1,102-row validation. Baseline macro-F1 0.4884; PI recall 20.77%; JB recall 41.76%; benign FPR 11.28%.
+467/1,102 errors occurred in all five fits. Source/label coupling and lexical/length shifts co-occur, so no sole cause is established.
+V8 is a 0-row source/label gate package; rights and independent adjudication remain open. Test/source-evaluation stayed closed; no L3 run.</x:v>
       </x:c>
       <x:c r="L6" s="6" t="inlineStr">
         <x:is>
@@ -909,7 +991,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="7" ht="110" customHeight="1">
+    <x:row r="7" ht="146" customHeight="1">
       <x:c r="A7" s="7" t="inlineStr">
         <x:is>
           <x:t>SE182087</x:t>
@@ -963,9 +1045,11 @@
 - Ngày 26/09: Báo cáo trực tiếp tại trường với GVHD ThS. Trần Văn Ninh; thuyết trình Phần 1 (Lỗ hổng ranh giới phẳng &amp; phân loại tấn công) và Phần 2 (Cơ sở lý thuyết, SOTA, Guardrail Trilemma).</x:t>
         </x:is>
       </x:c>
-      <x:c r="J7" s="7" t="str">
-        <x:v>Review 1: snapshot 03/10; hoàn tất 04/10 theo xác nhận.
-Report 1/2 đã ghi hoàn thành; chưa có chứng cứ gửi GVHD. Không phải nghiệm thu mô hình.</x:v>
+      <x:c r="J7" s="7" t="inlineStr">
+        <x:is>
+          <x:t>Review 1: snapshot 03/10; hoàn tất 04/10 theo xác nhận.
+Report 1/2 đã ghi hoàn thành; chưa có chứng cứ gửi GVHD. Không phải nghiệm thu mô hình.</x:t>
+        </x:is>
       </x:c>
       <x:c r="K7" s="7" t="inlineStr">
         <x:is>
@@ -1056,7 +1140,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="8" ht="110" customHeight="1">
+    <x:row r="8" ht="146" customHeight="1">
       <x:c r="A8" s="6" t="inlineStr">
         <x:is>
           <x:t>SE181851</x:t>
@@ -1110,9 +1194,11 @@
 - Ngày 26/09: Báo cáo trực tiếp tại trường với GVHD ThS. Trần Văn Ninh; thuyết trình Phần 3 (Kết quả thực nghiệm đối chuẩn chéo D1–D6 chỉ ra các failure modes y văn).</x:t>
         </x:is>
       </x:c>
-      <x:c r="J8" s="6" t="str">
-        <x:v>Review 1: snapshot 03/10; hoàn tất 04/10 theo xác nhận.
-Report 1/2 đã ghi hoàn thành; chưa có chứng cứ gửi GVHD. Không phải nghiệm thu mô hình.</x:v>
+      <x:c r="J8" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Review 1: snapshot 03/10; hoàn tất 04/10 theo xác nhận.
+Report 1/2 đã ghi hoàn thành; chưa có chứng cứ gửi GVHD. Không phải nghiệm thu mô hình.</x:t>
+        </x:is>
       </x:c>
       <x:c r="K8" s="6" t="inlineStr">
         <x:is>
@@ -1203,7 +1289,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="9" ht="110" customHeight="1">
+    <x:row r="9" ht="158" customHeight="1">
       <x:c r="A9" s="7" t="inlineStr">
         <x:is>
           <x:t>SE180235</x:t>
@@ -1258,9 +1344,11 @@
 - Hỗ trợ rà soát docs Chapter 1 &amp; 2.</x:t>
         </x:is>
       </x:c>
-      <x:c r="J9" s="7" t="str">
-        <x:v>Review 1: snapshot 03/10; hoàn tất 04/10 theo xác nhận.
-Report 1/2 đã ghi hoàn thành; chưa có chứng cứ gửi GVHD. Không phải nghiệm thu mô hình.</x:v>
+      <x:c r="J9" s="7" t="inlineStr">
+        <x:is>
+          <x:t>Review 1: snapshot 03/10; hoàn tất 04/10 theo xác nhận.
+Report 1/2 đã ghi hoàn thành; chưa có chứng cứ gửi GVHD. Không phải nghiệm thu mô hình.</x:t>
+        </x:is>
       </x:c>
       <x:c r="K9" s="7" t="inlineStr">
         <x:is>
@@ -1355,8 +1443,8 @@
   <x:mergeCells count="7">
     <x:mergeCell ref="B4:B5"/>
     <x:mergeCell ref="A2:U2"/>
+    <x:mergeCell ref="C4:F4"/>
     <x:mergeCell ref="A4:A5"/>
-    <x:mergeCell ref="C4:F4"/>
     <x:mergeCell ref="A1:U1"/>
     <x:mergeCell ref="G4:U4"/>
     <x:mergeCell ref="A3:U3"/>
@@ -1471,7 +1559,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="6" ht="25" customHeight="1">
+    <x:row r="6" ht="38" customHeight="1">
       <x:c r="A6" s="9" t="inlineStr">
         <x:is>
           <x:t>T02</x:t>
@@ -1497,8 +1585,10 @@
           <x:t>Trường &amp; Đức</x:t>
         </x:is>
       </x:c>
-      <x:c r="F6" s="10" t="str">
-        <x:v>Final-Report/Meeting/Meeting 3_08_09_26.md</x:v>
+      <x:c r="F6" s="10" t="inlineStr">
+        <x:is>
+          <x:t>Final-Report/Meeting/Meeting 3_08_09_26.md</x:t>
+        </x:is>
       </x:c>
       <x:c r="G6" s="9" t="inlineStr">
         <x:is>
@@ -1876,7 +1966,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="17" ht="25" customHeight="1">
+    <x:row r="17" ht="38" customHeight="1">
       <x:c r="A17" s="9" t="inlineStr">
         <x:is>
           <x:t>T13</x:t>
@@ -1976,14 +2066,18 @@
           <x:t>Trường (Leader)</x:t>
         </x:is>
       </x:c>
-      <x:c r="F19" s="10" t="str">
-        <x:v>PI_GUARD_PROCESS_REPORT.xlsx</x:v>
-      </x:c>
-      <x:c r="G19" s="9" t="str">
-        <x:v>03/10/2026</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="60" customHeight="1">
+      <x:c r="F19" s="10" t="inlineStr">
+        <x:is>
+          <x:t>PI_GUARD_PROCESS_REPORT.xlsx</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G19" s="9" t="inlineStr">
+        <x:is>
+          <x:t>03/10/2026</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="62" customHeight="1">
       <x:c r="A20" s="9" t="inlineStr">
         <x:is>
           <x:t>T16</x:t>
@@ -1994,19 +2088,25 @@
           <x:t>Tuần 4 (28/09 - 04/10)</x:t>
         </x:is>
       </x:c>
-      <x:c r="C20" s="10" t="str">
-        <x:v>CỘT MỐC 1 — REVIEW 1 HOÀN TẤT NGÀY 04/10/2026 (theo xác nhận của người dùng)</x:v>
-      </x:c>
-      <x:c r="D20" s="15" t="str">
-        <x:v>Hoàn thành</x:v>
+      <x:c r="C20" s="10" t="inlineStr">
+        <x:is>
+          <x:t>CỘT MỐC 1 — REVIEW 1 HOÀN TẤT NGÀY 04/10/2026 (theo xác nhận của người dùng)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D20" s="15" t="inlineStr">
+        <x:is>
+          <x:t>Hoàn thành</x:t>
+        </x:is>
       </x:c>
       <x:c r="E20" s="10" t="inlineStr">
         <x:is>
           <x:t>Cả 4 thành viên</x:t>
         </x:is>
       </x:c>
-      <x:c r="F20" s="10" t="str">
-        <x:v>workspaces/truongnv/reports/report_for_review1/REVIEW_1_COMPLETION_REPORT_2026-10-04.md (báo cáo tiến độ, không phải biên bản nghiệm thu mô hình)</x:v>
+      <x:c r="F20" s="10" t="inlineStr">
+        <x:is>
+          <x:t>workspaces/truongnv/reports/report_for_review1/REVIEW_1_COMPLETION_REPORT_2026-10-04.md (báo cáo tiến độ, không phải biên bản nghiệm thu mô hình)</x:t>
+        </x:is>
       </x:c>
       <x:c r="G20" s="9" t="inlineStr">
         <x:is>
@@ -2014,7 +2114,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="21" ht="25" customHeight="1">
+    <x:row r="21" ht="100" customHeight="1">
       <x:c r="A21" s="9" t="inlineStr">
         <x:is>
           <x:t>T17</x:t>
@@ -2025,12 +2125,14 @@
           <x:t>Tuần 5 - 6 (05/10 - 18/10)</x:t>
         </x:is>
       </x:c>
-      <x:c r="C21" s="10" t="str">
-        <x:v>Duyệt nguồn/nhãn; group-aware split; fit baseline TF-IDF ba lớp</x:v>
+      <x:c r="C21" s="10" t="inlineStr">
+        <x:is>
+          <x:t>Duyệt nguồn/nhãn; group-aware split; fit baseline TF-IDF ba lớp</x:t>
+        </x:is>
       </x:c>
       <x:c r="D21" s="13" t="inlineStr">
         <x:is>
-          <x:t>Chưa bắt đầu</x:t>
+          <x:t>Đang thực hiện</x:t>
         </x:is>
       </x:c>
       <x:c r="E21" s="10" t="inlineStr">
@@ -2038,13 +2140,13 @@
           <x:t>Trường &amp; Đức</x:t>
         </x:is>
       </x:c>
-      <x:c r="F21" s="10" t="str">
-        <x:v>L2 model + metrics</x:v>
-      </x:c>
-      <x:c r="G21" s="9" t="inlineStr">
-        <x:is>
-          <x:t>18/10/2026</x:t>
-        </x:is>
+      <x:c r="F21" s="10" t="inlineStr">
+        <x:is>
+          <x:t>L2 model + metrics</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G21" s="19" t="str">
+        <x:v>V7.1 L2 done: five fits; weak validation. Rights/labels open; V8 has 0 rows. No test/source-eval or L3.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="25" customHeight="1">
@@ -2058,8 +2160,10 @@
           <x:t>Tuần 7 (19/10 - 25/10)</x:t>
         </x:is>
       </x:c>
-      <x:c r="C22" s="10" t="str">
-        <x:v>Fine-tune DeBERTa; tích hợp demo L2/L3; soạn Chapter 3 và slide</x:v>
+      <x:c r="C22" s="10" t="inlineStr">
+        <x:is>
+          <x:t>Fine-tune DeBERTa; tích hợp demo L2/L3; soạn Chapter 3 và slide</x:t>
+        </x:is>
       </x:c>
       <x:c r="D22" s="13" t="inlineStr">
         <x:is>
@@ -2071,8 +2175,10 @@
           <x:t>Đức &amp; Trường</x:t>
         </x:is>
       </x:c>
-      <x:c r="F22" s="10" t="str">
-        <x:v>Checkpoint; inference thật; tài liệu Review 2</x:v>
+      <x:c r="F22" s="10" t="inlineStr">
+        <x:is>
+          <x:t>Checkpoint; inference thật; tài liệu Review 2</x:t>
+        </x:is>
       </x:c>
       <x:c r="G22" s="9" t="inlineStr">
         <x:is>
@@ -2091,8 +2197,10 @@
           <x:t>Tuần 8 (26/10 - 01/11)</x:t>
         </x:is>
       </x:c>
-      <x:c r="C23" s="10" t="str">
-        <x:v>Review 2: Chapter 3 và demo model PI-Guard ba nhãn</x:v>
+      <x:c r="C23" s="10" t="inlineStr">
+        <x:is>
+          <x:t>Review 2: Chapter 3 và demo model PI-Guard ba nhãn</x:t>
+        </x:is>
       </x:c>
       <x:c r="D23" s="13" t="inlineStr">
         <x:is>
@@ -2104,8 +2212,10 @@
           <x:t>Cả 4 thành viên</x:t>
         </x:is>
       </x:c>
-      <x:c r="F23" s="10" t="str">
-        <x:v>Demo thật, provenance và checklist trạng thái</x:v>
+      <x:c r="F23" s="10" t="inlineStr">
+        <x:is>
+          <x:t>Demo thật, provenance và checklist trạng thái</x:t>
+        </x:is>
       </x:c>
       <x:c r="G23" s="9" t="inlineStr">
         <x:is>
@@ -2124,8 +2234,10 @@
           <x:t>Tuần 9 - 10 (02/11 - 15/11)</x:t>
         </x:is>
       </x:c>
-      <x:c r="C24" s="10" t="str">
-        <x:v>Đánh giá robustness DeBERTa; hoàn tất Report No.4</x:v>
+      <x:c r="C24" s="10" t="inlineStr">
+        <x:is>
+          <x:t>Đánh giá robustness DeBERTa; hoàn tất Report No.4</x:t>
+        </x:is>
       </x:c>
       <x:c r="D24" s="13" t="inlineStr">
         <x:is>
@@ -2137,8 +2249,10 @@
           <x:t>Việt &amp; Đức</x:t>
         </x:is>
       </x:c>
-      <x:c r="F24" s="10" t="str">
-        <x:v>Report No.4; metrics từng lớp; checkpoint/hash</x:v>
+      <x:c r="F24" s="10" t="inlineStr">
+        <x:is>
+          <x:t>Report No.4; metrics từng lớp; checkpoint/hash</x:t>
+        </x:is>
       </x:c>
       <x:c r="G24" s="9" t="inlineStr">
         <x:is>
@@ -2220,7 +2334,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="27" ht="25" customHeight="1">
+    <x:row r="27" ht="38" customHeight="1">
       <x:c r="A27" s="9" t="inlineStr">
         <x:is>
           <x:t>T23</x:t>
@@ -2481,16 +2595,20 @@
           <x:t>Đánh giá kết quả nghiên cứu và thống nhất slide báo cáo tiến độ gặp GVHD ngày 10/09/2026.</x:t>
         </x:is>
       </x:c>
-      <x:c r="F7" s="10" t="str">
-        <x:v>Trường và Đức hoàn thiện bộ slide 22 trang; Việt và Phương rà soát, không có ý kiến bổ sung.
-Đầu ra: Meeting 3_08_09_26.md; slide đã gỡ ngày 08/10/2026.</x:v>
-      </x:c>
-      <x:c r="G7" s="14" t="str">
-        <x:v>Hoàn thành (100%)
-Final-Report/Meeting/Meeting 3_08_09_26.md</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="80" customHeight="1">
+      <x:c r="F7" s="10" t="inlineStr">
+        <x:is>
+          <x:t>Trường và Đức hoàn thiện bộ slide 22 trang; Việt và Phương rà soát, không có ý kiến bổ sung.
+Đầu ra: Meeting 3_08_09_26.md; slide đã gỡ ngày 08/10/2026.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G7" s="14" t="inlineStr">
+        <x:is>
+          <x:t>Hoàn thành (100%)
+Final-Report/Meeting/Meeting 3_08_09_26.md</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="98" customHeight="1">
       <x:c r="A8" s="9" t="inlineStr">
         <x:is>
           <x:t>Meet 04</x:t>
@@ -2529,7 +2647,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="9" ht="80" customHeight="1">
+    <x:row r="9" ht="86" customHeight="1">
       <x:c r="A9" s="9" t="inlineStr">
         <x:is>
           <x:t>Meet 05</x:t>
@@ -2568,7 +2686,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="10" ht="80" customHeight="1">
+    <x:row r="10" ht="98" customHeight="1">
       <x:c r="A10" s="9" t="inlineStr">
         <x:is>
           <x:t>Meet 06</x:t>

</xml_diff>